<commit_message>
Make 2-column table value text always #000000
Per explicit instruction: table value-column text is #000000 always,
not #333333 as NOTIFICATION_STANDARDS.md previously specified. Label
column stays #666666 (muted gray) and general paragraph body copy
elsewhere is unaffected (#333333 is correct there) — this only touches
table <td> value cells (identified by their 82.7863% width).

Updated the 3 files with tables fixed since the standards doc landed
(additional_comment_added, change_request_approval, order_delivered),
the standards doc itself and its reconciliation note, the working
transform script's default, and regenerated 78Sample_updated.xlsx.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011We9gy6ZLYcTcTQxPWoR4Y
</commit_message>
<xml_diff>
--- a/servicenow/email_notifications/78Sample_updated.xlsx
+++ b/servicenow/email_notifications/78Sample_updated.xlsx
@@ -521,7 +521,7 @@
 &lt;tbody&gt;
 &lt;tr&gt;
 &lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #666666; width: 17.2137%; padding: 0 20px 8px 0; vertical-align: top; white-space: nowrap;" valign="top"&gt;Short Description:&lt;/td&gt;
-&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #333333; line-height: 1.5; width: 82.7863%; padding: 0 0 8px 0; vertical-align: top;" valign="top"&gt;${short_description}&lt;/td&gt;
+&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5; width: 82.7863%; padding: 0 0 8px 0; vertical-align: top;" valign="top"&gt;${short_description}&lt;/td&gt;
 &lt;/tr&gt;
 &lt;/tbody&gt;
 &lt;/table&gt;
@@ -608,8 +608,8 @@
 &lt;p style="margin: 0 0 24px 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #333333; line-height: 1.5;"&gt;Please review the change ${mail_script:nvidia_change_record_link} by ${sysapproval.opened_by.name}. After your review, select the appropriate link below and reply.&lt;/p&gt;
 &lt;!-- 2-column tabular content --&gt;
 &lt;table role="presentation" border="0" width="100%" cellspacing="0" cellpadding="0" style="margin: 0 0 24px 0;"&gt;
-&lt;tr&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #666666; width: 17.2137%; padding: 0 20px 8px 0; vertical-align: top; white-space: nowrap;"&gt;Short Description:&lt;/td&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #333333; width: 82.7863%; padding: 0 0 8px 0; vertical-align: top;"&gt;${sysapproval.short_description}&lt;/td&gt;&lt;/tr&gt;
-&lt;tr&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #666666; width: 17.2137%; padding: 0 20px 8px 0; vertical-align: top; white-space: nowrap;"&gt;Justification:&lt;/td&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #333333; width: 82.7863%; padding: 0 0 8px 0; vertical-align: top;"&gt;${sysapproval.justification}&lt;/td&gt;&lt;/tr&gt;
+&lt;tr&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #666666; width: 17.2137%; padding: 0 20px 8px 0; vertical-align: top; white-space: nowrap;"&gt;Short Description:&lt;/td&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; width: 82.7863%; padding: 0 0 8px 0; vertical-align: top;"&gt;${sysapproval.short_description}&lt;/td&gt;&lt;/tr&gt;
+&lt;tr&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #666666; width: 17.2137%; padding: 0 20px 8px 0; vertical-align: top; white-space: nowrap;"&gt;Justification:&lt;/td&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; width: 82.7863%; padding: 0 0 8px 0; vertical-align: top;"&gt;${sysapproval.justification}&lt;/td&gt;&lt;/tr&gt;
 &lt;/table&gt;
 &lt;!-- CTA Buttons --&gt;
 &lt;table border="0" cellspacing="0" cellpadding="0"&gt;

</xml_diff>

<commit_message>
Make all non-link text #000000 — drop #333333 and #666666 entirely
Per explicit instruction: no body/label text should be #666666 or
#333333 anywhere. This affects every notification fixed since
NOTIFICATION_STANDARDS.md landed (they'd used #333333 for general body
copy and #666666 for the table label column / footer, matching what
that doc originally specified). Only links keep their green.

Updated: additional_comment_added, change_request_approval,
incident_resolved, nvidia_access_reinstatement_instructions,
order_delivered, requested_item_closed, requested_item_commented.

Also updated NOTIFICATION_STANDARDS.md (typography rule, footer color,
table label/value colors, reconciliation table) and the working
transform script's defaults so this applies automatically going
forward, and regenerated 78Sample_updated.xlsx.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011We9gy6ZLYcTcTQxPWoR4Y
</commit_message>
<xml_diff>
--- a/servicenow/email_notifications/78Sample_updated.xlsx
+++ b/servicenow/email_notifications/78Sample_updated.xlsx
@@ -514,13 +514,13 @@
           <t>&lt;!-- Email Heading --&gt;
 &lt;h1 style="margin: 0 0 24px 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 24px; font-weight: bold; color: #000000; line-height: 1.3;"&gt;New Comment on ${number}&lt;/h1&gt;
 &lt;!-- Greeting --&gt;
-&lt;p style="margin: 0 0 24px 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #333333; line-height: 1.5;"&gt;Hello ${caller_id.first_name},&lt;/p&gt;
-&lt;p style="margin: 0 0 24px 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #333333; line-height: 1.5;"&gt;You received a new comment on your incident.&lt;/p&gt;
+&lt;p style="margin: 0 0 24px 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;Hello ${caller_id.first_name},&lt;/p&gt;
+&lt;p style="margin: 0 0 24px 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;You received a new comment on your incident.&lt;/p&gt;
 &lt;!-- 2-column tabular content --&gt;
 &lt;table role="presentation" border="0" width="100%" cellspacing="0" cellpadding="0" style="margin: 0 0 24px 0;"&gt;
 &lt;tbody&gt;
 &lt;tr&gt;
-&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #666666; width: 17.2137%; padding: 0 20px 8px 0; vertical-align: top; white-space: nowrap;" valign="top"&gt;Short Description:&lt;/td&gt;
+&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; width: 17.2137%; padding: 0 20px 8px 0; vertical-align: top; white-space: nowrap;" valign="top"&gt;Short Description:&lt;/td&gt;
 &lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5; width: 82.7863%; padding: 0 0 8px 0; vertical-align: top;" valign="top"&gt;${short_description}&lt;/td&gt;
 &lt;/tr&gt;
 &lt;/tbody&gt;
@@ -528,7 +528,7 @@
 &lt;!-- Comment label --&gt;
 &lt;p style="margin: 0 0 8px 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: bold; color: #000000; line-height: 1.5;"&gt;Comment:&lt;/p&gt;
 &lt;!-- Comment body — rendered by mail script --&gt;
-&lt;p style="margin: 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #333333; line-height: 1.5;"&gt;${mail_script:it_single_comment_clean}&lt;/p&gt;</t>
+&lt;p style="margin: 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;${mail_script:it_single_comment_clean}&lt;/p&gt;</t>
         </is>
       </c>
     </row>
@@ -604,12 +604,12 @@
         <is>
           <t>&lt;!-- Email Heading --&gt;
 &lt;h1 style="margin: 0 0 24px 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 24px; font-weight: bold; color: #000000; line-height: 1.3;"&gt;Change request approval needed&lt;/h1&gt;
-&lt;p style="margin: 0 0 24px 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #333333; line-height: 1.5;"&gt;Hello ${approver.name},&lt;/p&gt;
-&lt;p style="margin: 0 0 24px 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #333333; line-height: 1.5;"&gt;Please review the change ${mail_script:nvidia_change_record_link} by ${sysapproval.opened_by.name}. After your review, select the appropriate link below and reply.&lt;/p&gt;
+&lt;p style="margin: 0 0 24px 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;Hello ${approver.name},&lt;/p&gt;
+&lt;p style="margin: 0 0 24px 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;Please review the change ${mail_script:nvidia_change_record_link} by ${sysapproval.opened_by.name}. After your review, select the appropriate link below and reply.&lt;/p&gt;
 &lt;!-- 2-column tabular content --&gt;
 &lt;table role="presentation" border="0" width="100%" cellspacing="0" cellpadding="0" style="margin: 0 0 24px 0;"&gt;
-&lt;tr&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #666666; width: 17.2137%; padding: 0 20px 8px 0; vertical-align: top; white-space: nowrap;"&gt;Short Description:&lt;/td&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; width: 82.7863%; padding: 0 0 8px 0; vertical-align: top;"&gt;${sysapproval.short_description}&lt;/td&gt;&lt;/tr&gt;
-&lt;tr&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #666666; width: 17.2137%; padding: 0 20px 8px 0; vertical-align: top; white-space: nowrap;"&gt;Justification:&lt;/td&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; width: 82.7863%; padding: 0 0 8px 0; vertical-align: top;"&gt;${sysapproval.justification}&lt;/td&gt;&lt;/tr&gt;
+&lt;tr&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; width: 17.2137%; padding: 0 20px 8px 0; vertical-align: top; white-space: nowrap;"&gt;Short Description:&lt;/td&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; width: 82.7863%; padding: 0 0 8px 0; vertical-align: top;"&gt;${sysapproval.short_description}&lt;/td&gt;&lt;/tr&gt;
+&lt;tr&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; width: 17.2137%; padding: 0 20px 8px 0; vertical-align: top; white-space: nowrap;"&gt;Justification:&lt;/td&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; width: 82.7863%; padding: 0 0 8px 0; vertical-align: top;"&gt;${sysapproval.justification}&lt;/td&gt;&lt;/tr&gt;
 &lt;/table&gt;
 &lt;!-- CTA Buttons --&gt;
 &lt;table border="0" cellspacing="0" cellpadding="0"&gt;
@@ -674,13 +674,13 @@
           <t>&lt;!-- Email Heading --&gt;
 &lt;h1 style="margin: 0 0 24px 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 24px; font-weight: bold; color: #000000; line-height: 1.3;"&gt;${number} Resolved&lt;/h1&gt;
 &lt;!-- Greeting --&gt;
-&lt;p style="margin: 0 0 24px 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #333333; line-height: 1.5;"&gt;Hello ${caller_id.first_name},&lt;/p&gt;
-&lt;p style="margin: 0 0 24px 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #333333; line-height: 1.5;"&gt;We are pleased to inform that your incident has been resolved.&lt;/p&gt;
-&lt;p style="margin: 0 0 24px 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #333333; line-height: 1.5;"&gt;If you are still having issues, you can reopen ${mail_script:link_to_portal_nvidia} within 7 days.&lt;/p&gt;
+&lt;p style="margin: 0 0 24px 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;Hello ${caller_id.first_name},&lt;/p&gt;
+&lt;p style="margin: 0 0 24px 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;We are pleased to inform that your incident has been resolved.&lt;/p&gt;
+&lt;p style="margin: 0 0 24px 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;If you are still having issues, you can reopen ${mail_script:link_to_portal_nvidia} within 7 days.&lt;/p&gt;
 &lt;!-- Survey intro + tertiary CTA — kept as an 8px-spaced pair, same as a
      comment label + comment body, since the link answers the sentence
      directly above it. --&gt;
-&lt;p style="margin: 0 0 8px 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #333333; line-height: 1.5;"&gt;Please take a short survey to rate your experience with IT.&lt;/p&gt;
+&lt;p style="margin: 0 0 8px 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;Please take a short survey to rate your experience with IT.&lt;/p&gt;
 &lt;p style="margin: 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: bold; color: #76b900; line-height: 1.5;"&gt;${mail_script:incident_survey_link_nvidia}&lt;/p&gt;</t>
         </is>
       </c>
@@ -705,10 +705,10 @@
         <is>
           <t>&lt;!-- Email Heading --&gt;
 &lt;h1 style="margin: 0 0 24px 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 24px; font-weight: bold; color: #000000; line-height: 1.3;"&gt;${number} has been closed&lt;/h1&gt;
-&lt;p style="margin: 0 0 24px 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #333333; line-height: 1.5;"&gt;Hello ${requested_for.first_name},&lt;/p&gt;
-&lt;p style="margin: 0 0 24px 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #333333; line-height: 1.5;"&gt;Good news -- ${mail_script:nvidia_uri_ref_styled} has been fulfilled.&lt;/p&gt;
-&lt;p style="margin: 0 0 24px 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #333333; line-height: 1.5;"&gt;You can report an issue within 7 days if it was not fulfilled to your satisfaction.&lt;/p&gt;
-&lt;p style="margin: 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #333333; line-height: 1.5;"&gt;Let us know how we're doing. &lt;a href="${mail_script:nvidia_survey_link}" style="color: #76b900; font-weight: bold; text-decoration: underline;"&gt;Share Your Feedback&lt;/a&gt;&lt;/p&gt;</t>
+&lt;p style="margin: 0 0 24px 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;Hello ${requested_for.first_name},&lt;/p&gt;
+&lt;p style="margin: 0 0 24px 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;Good news -- ${mail_script:nvidia_uri_ref_styled} has been fulfilled.&lt;/p&gt;
+&lt;p style="margin: 0 0 24px 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;You can report an issue within 7 days if it was not fulfilled to your satisfaction.&lt;/p&gt;
+&lt;p style="margin: 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;Let us know how we're doing. &lt;a href="${mail_script:nvidia_survey_link}" style="color: #76b900; font-weight: bold; text-decoration: underline;"&gt;Share Your Feedback&lt;/a&gt;&lt;/p&gt;</t>
         </is>
       </c>
     </row>
@@ -732,12 +732,12 @@
         <is>
           <t>&lt;!-- Email Heading --&gt;
 &lt;h1 style="margin: 0 0 24px 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 24px; font-weight: bold; color: #000000; line-height: 1.3;"&gt;A comment was added to ${cat_item.number}&lt;/h1&gt;
-&lt;p style="margin: 0 0 24px 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #333333; line-height: 1.5;"&gt;Hello ${requested_for.first_name},&lt;/p&gt;
-&lt;p style="margin: 0 0 24px 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #333333; line-height: 1.5;"&gt;See comment details for ${mail_script:nvidia_uri_ref_styled} below.&lt;/p&gt;
+&lt;p style="margin: 0 0 24px 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;Hello ${requested_for.first_name},&lt;/p&gt;
+&lt;p style="margin: 0 0 24px 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;See comment details for ${mail_script:nvidia_uri_ref_styled} below.&lt;/p&gt;
 &lt;!-- Comment label --&gt;
 &lt;p style="margin: 0 0 8px 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: bold; color: #000000; line-height: 1.5;"&gt;Comment:&lt;/p&gt;
 &lt;!-- Comment body — rendered by mail script --&gt;
-&lt;p style="margin: 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #333333; line-height: 1.5;"&gt;${mail_script:it_single_comment_clean}&lt;/p&gt;</t>
+&lt;p style="margin: 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;${mail_script:it_single_comment_clean}&lt;/p&gt;</t>
         </is>
       </c>
     </row>

</xml_diff>